<commit_message>
updated full review process
</commit_message>
<xml_diff>
--- a/changelog/v3.2.1/claude_review/Internal Peer Checklist - X1_IOB_v3.2.1 (Claude).xlsx
+++ b/changelog/v3.2.1/claude_review/Internal Peer Checklist - X1_IOB_v3.2.1 (Claude).xlsx
@@ -1584,7 +1584,11 @@
       <c r="D21" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="E21" s="1"/>
+      <c r="E21" s="1" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
       <c r="F21">
         <f t="shared" si="0"/>
         <v>1</v>
@@ -1592,6 +1596,11 @@
       <c r="G21" t="str">
         <f t="shared" si="1"/>
         <v/>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Full 10-sheet port audit vs. X1_IO V3.0.1 20180224.pdf (2018 PADS ref, several revisions old): all major blocks present, refdes match almost 1:1 across ~500+ components. See claude_review/REVIEW_IOB_v3.2.1.md.</t>
+        </is>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.35">
@@ -1601,7 +1610,11 @@
       <c r="D22" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="E22" s="1"/>
+      <c r="E22" s="1" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
       <c r="F22">
         <f t="shared" si="0"/>
         <v>1</v>
@@ -1609,6 +1622,11 @@
       <c r="G22" t="str">
         <f t="shared" si="1"/>
         <v/>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Same audit, corrected after re-verification: U6 pin35/36 ADC renames (changelog items 6/7) confirmed exact match, same mux chips (U9/U28/U35) in both revisions, only output names changed. 1 remaining unexplained item: U29/U33 marked HTC MC34063AD vs. 2018's NCP3063 -- plausible sourcing substitution, predates v3.2.0 baseline, flagged for engineer confirmation, not blocking.</t>
+        </is>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.35">
@@ -1644,7 +1662,11 @@
       <c r="D24" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="E24" s="1"/>
+      <c r="E24" s="1" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
       <c r="F24">
         <f t="shared" si="0"/>
         <v>1</v>
@@ -1652,6 +1674,11 @@
       <c r="G24" t="str">
         <f t="shared" si="1"/>
         <v/>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>U6 pad 35=ADC_B, pad 36=ADC_D, pad 69/70=unconnected -- confirmed directly via tools/kicad-query/pcb_net.py against IOB_v3.2.1.kicad_pcb, exact match to changelog items 6/7/9/10</t>
+        </is>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.35">
@@ -2333,7 +2360,11 @@
       <c r="D20" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="E20" s="1"/>
+      <c r="E20" s="1" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
       <c r="F20">
         <f t="shared" si="0"/>
         <v>1</v>
@@ -2341,6 +2372,11 @@
       <c r="G20" t="str">
         <f t="shared" si="0"/>
         <v/>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>ADF logo present on top silkscreen (tools/kicad-reports render, --side top)</t>
+        </is>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.35">
@@ -2350,7 +2386,11 @@
       <c r="D22" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="E22" s="1"/>
+      <c r="E22" s="1" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
       <c r="F22">
         <f t="shared" si="0"/>
         <v>1</v>
@@ -2358,6 +2398,11 @@
       <c r="G22" t="str">
         <f t="shared" si="0"/>
         <v/>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Silkscreen under ADF logo reads 'IOB_V1.0' -- stale, this is revision v3.2.1. Confirmed by cropping tools/kicad-reports board render (--side top) at 4x. Needs a silkscreen text update, not just a title-block field.</t>
+        </is>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.35">
@@ -2691,7 +2736,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>IOB/Gerber/ has NO F_Cu/B_Cu (copper) gerbers at all -- board is not fabricable as committed</t>
+          <t>IOB/Gerber/ has no F_Cu/B_Cu, but a complete copper export DOES exist for v3.2.1 (changelog/v3.2.1/gerber_v3.2.1_v.3.2.0/TOP_new.pho, BOTTOM_new.pho -- real, ~70k-command gerbers, exported via gerbv). IOB/Gerber/ just wasn't synced with it -- ask engineer whether that folder is meant to hold the full set.</t>
         </is>
       </c>
     </row>
@@ -2769,7 +2814,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>IOB/Gerber/ has NO F_Paste/B_Paste gerbers</t>
+          <t>IOB/Gerber/ has no F_Paste/B_Paste, but Paste_top_new.pho/Paste_bottom_new.pho (same diff folder) confirm a complete paste export exists for v3.2.1. Same sync question as row 46.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
updated claude review on BOM comparison
</commit_message>
<xml_diff>
--- a/changelog/v3.2.1/claude_review/Internal Peer Checklist - X1_IOB_v3.2.1 (Claude).xlsx
+++ b/changelog/v3.2.1/claude_review/Internal Peer Checklist - X1_IOB_v3.2.1 (Claude).xlsx
@@ -1625,7 +1625,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Same audit, corrected after re-verification: U6 pin35/36 ADC renames (changelog items 6/7) confirmed exact match, same mux chips (U9/U28/U35) in both revisions, only output names changed. 1 remaining unexplained item: U29/U33 marked HTC MC34063AD vs. 2018's NCP3063 -- plausible sourcing substitution, predates v3.2.0 baseline, flagged for engineer confirmation, not blocking.</t>
+          <t>Corrected after re-verification with the actual v3.2.0 BOM (user-provided, IOB_BOM_v3.2.0_2022.xlsx): 535/535 populated refdes match exactly between v3.2.0 and v3.2.1 (only DNP-scope difference, fully explained). U6 pin35/36 ADC renames (items 6/7) confirmed exact match. U29/U33 HTC MC34063AD confirmed already present in 2022 -- not a migration change, no open items from this audit.</t>
         </is>
       </c>
     </row>
@@ -1780,7 +1780,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>C32 not marked DNP: schematic symbol dnp=no, BOM value has no ';DNI' suffix, no PCB footprint attr -- but changelog item 12 states 'C32, D48, D51 are now DNI/DNP'. D48/D51 ARE correctly dnp=yes. Confirm with engineer whether C32 should be DNP or the changelog is wrong.</t>
+          <t>C32 not marked DNP: schematic symbol dnp=no, drawn with a visual DNI cross-out but property never set, BOM value has no ';DNI' suffix, no PCB footprint attr, AND the actual v3.2.0 production BOM (IOB_BOM_v3.2.0_2022.xlsx) shows C32 as a normal populated part too -- 4 independent sources agree it has never been DNP. D48/D51 ARE correctly dnp=yes. Confirm with engineer whether C32 should be DNP.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
updated after challenge on C32 issue
</commit_message>
<xml_diff>
--- a/changelog/v3.2.1/claude_review/Internal Peer Checklist - X1_IOB_v3.2.1 (Claude).xlsx
+++ b/changelog/v3.2.1/claude_review/Internal Peer Checklist - X1_IOB_v3.2.1 (Claude).xlsx
@@ -1780,7 +1780,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>C32 not marked DNP: schematic symbol dnp=no, drawn with a visual DNI cross-out but property never set, BOM value has no ';DNI' suffix, no PCB footprint attr, AND the actual v3.2.0 production BOM (IOB_BOM_v3.2.0_2022.xlsx) shows C32 as a normal populated part too -- 4 independent sources agree it has never been DNP. D48/D51 ARE correctly dnp=yes. Confirm with engineer whether C32 should be DNP.</t>
+          <t>Corrected 2026-08-19: earlier claim that the schematic visually draws C32 DNP was a misread -- the red X/DNI mark actually belongs to C8 (adjacent, same value/footprint, easy to conflate at low res). C32 itself is a normal populated part everywhere (schematic dnp=no, PCB, current BOM, and the real v3.2.0 BOM). D48/D51 correctly dnp=yes. Changelog item 12 most likely means C8, not C32 -- a documentation typo, not a PCB defect. Still NO on literal text match since changelog says C32.</t>
         </is>
       </c>
     </row>
@@ -2564,7 +2564,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Same C32 DNP discrepancy as schematic checklist row 30 -- footprint has no dnp/exclude attribute set on the PCB side either, contradicting changelog item 12</t>
+          <t>Corrected 2026-08-19: same C32/C8 mixup as schematic checklist row 30 -- C32 was never DNP on the PCB either; C8 is the actual DNP part and has been since at least v3.2.0. Likely a changelog typo (C32 should read C8), not a real PCB update gap.</t>
         </is>
       </c>
     </row>

</xml_diff>